<commit_message>
Data cleaning done and final dataset created
</commit_message>
<xml_diff>
--- a/Outputs&ExcelFiles/FinalBigDataSet.xlsx
+++ b/Outputs&ExcelFiles/FinalBigDataSet.xlsx
@@ -1805,7 +1805,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>$50</t>
+          <t>$50,000,000</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>$175</t>
+          <t>$175,000,000</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>$90</t>
+          <t>$90,000,000</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>$17</t>
+          <t>$17,000,000</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4843,7 +4843,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$11,000,000</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>$8</t>
+          <t>$8,000,000</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -5959,7 +5959,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15,000,000</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -6827,7 +6827,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>$22</t>
+          <t>$22,000,000</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -7385,7 +7385,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>$1</t>
+          <t>$1,300,000</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>$13</t>
+          <t>$13,000,000</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -7633,7 +7633,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,300,000</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -7695,7 +7695,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>$70</t>
+          <t>$70,000,000</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>$26</t>
+          <t>$26,000,000</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>$24</t>
+          <t>$24,000,000</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -8377,7 +8377,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -8439,7 +8439,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -8563,7 +8563,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -8687,7 +8687,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -9057,7 +9057,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>$13</t>
+          <t>$13,000,000</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -9119,7 +9119,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>$40</t>
+          <t>$40,000,000</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -9429,7 +9429,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$11,000,000</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -9553,7 +9553,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,000,000</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -9615,7 +9615,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15,000,000</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -9677,7 +9677,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,000,000</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -9739,7 +9739,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>$9</t>
+          <t>$9,600,000</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -9801,7 +9801,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>$19</t>
+          <t>$19,000,000</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -9863,7 +9863,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -10111,7 +10111,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,000,000</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -10235,7 +10235,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,400,000</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -10359,7 +10359,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t>$200,000,000</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -10669,7 +10669,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>$150</t>
+          <t>$150,000,000</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -12961,7 +12961,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15,000,000</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -13147,7 +13147,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>$110</t>
+          <t>$110,000,000</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -13209,7 +13209,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>$75</t>
+          <t>$90,000,000</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>$35</t>
+          <t>$35,000,000</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
@@ -14201,7 +14201,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -14697,7 +14697,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>$40</t>
+          <t>$40,000,000</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
@@ -15751,7 +15751,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>$50</t>
+          <t>$50,000,000</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -15875,7 +15875,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>$70</t>
+          <t>$70,000,000</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -16495,7 +16495,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>$40</t>
+          <t>$40,000,000</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -16681,7 +16681,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -16929,7 +16929,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -16991,7 +16991,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -17053,7 +17053,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>$13</t>
+          <t>$13,000,000</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -17177,7 +17177,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -17239,7 +17239,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>$7</t>
+          <t>$7,000,000</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -17425,7 +17425,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>$28</t>
+          <t>$28,000,000</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -17549,7 +17549,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>$31</t>
+          <t>$31,500,000</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -17611,7 +17611,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -17673,7 +17673,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>$1</t>
+          <t>$1,000,000</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -17797,7 +17797,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,000,000</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -17921,7 +17921,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$11,800,000</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -17983,7 +17983,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -18107,7 +18107,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -18169,7 +18169,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15,000,000</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -18231,7 +18231,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -18355,7 +18355,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>$4</t>
+          <t>$4,000,000</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -18417,7 +18417,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>$22</t>
+          <t>$22,500,000</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -18479,7 +18479,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>$6</t>
+          <t>$6,000,000</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -18541,7 +18541,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -18603,7 +18603,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -18665,7 +18665,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,000,000</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -18851,7 +18851,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -18913,7 +18913,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>$13</t>
+          <t>$13,000,000</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -18973,7 +18973,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>$35</t>
+          <t>$35,000,000</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -19097,7 +19097,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>$18</t>
+          <t>$18,500,000</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
@@ -19159,7 +19159,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>$1</t>
+          <t>$1,500,000</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -19345,7 +19345,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -19407,7 +19407,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,000,000</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
@@ -19469,7 +19469,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -19591,7 +19591,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -19653,7 +19653,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,500,000</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
@@ -19777,7 +19777,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>$13</t>
+          <t>$13,000,000</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
@@ -19839,7 +19839,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -19963,7 +19963,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -20025,7 +20025,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -20087,7 +20087,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>$40</t>
+          <t>$40,000,000</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -20149,7 +20149,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>$13</t>
+          <t>$13,000,000</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -20211,7 +20211,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
@@ -20273,7 +20273,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>$7</t>
+          <t>$7,500,000</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
@@ -20335,7 +20335,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,500,000</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -20397,7 +20397,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>$35</t>
+          <t>$35,000,000</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
@@ -21017,7 +21017,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>$300</t>
+          <t>$300,000,000</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
@@ -21203,7 +21203,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>$175</t>
+          <t>$175,000,000</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
@@ -21451,7 +21451,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>$125</t>
+          <t>$125,000,000</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
@@ -21761,7 +21761,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>$175</t>
+          <t>$175,000,000</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
@@ -21947,7 +21947,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>$149</t>
+          <t>$149,000,000</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
@@ -23249,7 +23249,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>$19</t>
+          <t>$19,300,000</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
@@ -23311,7 +23311,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>$70</t>
+          <t>$70,000,000</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
@@ -23435,7 +23435,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
@@ -23497,7 +23497,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
@@ -23621,7 +23621,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>$12</t>
+          <t>$12,000,000</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
@@ -23931,7 +23931,7 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
@@ -24489,7 +24489,7 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
@@ -25171,7 +25171,7 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>$125</t>
+          <t>$125,000,000</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
@@ -25233,7 +25233,7 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>$22</t>
+          <t>$22,000,000</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
@@ -25295,7 +25295,7 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
@@ -26039,7 +26039,7 @@
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t>$50</t>
+          <t>$50,000,000</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
@@ -26287,7 +26287,7 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>$21</t>
+          <t>$21,000,000</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
@@ -26533,7 +26533,7 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
@@ -26595,7 +26595,7 @@
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
@@ -26967,7 +26967,7 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
@@ -27029,7 +27029,7 @@
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
@@ -27277,7 +27277,7 @@
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,000,000</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
@@ -27401,7 +27401,7 @@
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
@@ -27463,7 +27463,7 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
@@ -27587,7 +27587,7 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>$7</t>
+          <t>$7,000,000</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
@@ -27897,7 +27897,7 @@
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
@@ -27959,7 +27959,7 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>$90</t>
+          <t>$90,000,000</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
@@ -28207,7 +28207,7 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>$60</t>
+          <t>$60,000,000</t>
         </is>
       </c>
       <c r="F449" t="inlineStr">
@@ -28269,7 +28269,7 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F450" t="inlineStr">
@@ -28703,7 +28703,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>$40</t>
+          <t>$40,000,000</t>
         </is>
       </c>
       <c r="F457" t="inlineStr">
@@ -28765,7 +28765,7 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>$31</t>
+          <t>$31,000,000</t>
         </is>
       </c>
       <c r="F458" t="inlineStr">
@@ -28889,7 +28889,7 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>$6</t>
+          <t>$6,500,000</t>
         </is>
       </c>
       <c r="F460" t="inlineStr">
@@ -29075,7 +29075,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F463" t="inlineStr">
@@ -29199,7 +29199,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>$7</t>
+          <t>$7,000,000</t>
         </is>
       </c>
       <c r="F465" t="inlineStr">
@@ -29261,7 +29261,7 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F466" t="inlineStr">
@@ -29323,7 +29323,7 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F467" t="inlineStr">
@@ -29445,7 +29445,7 @@
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>$43</t>
+          <t>$43,000,000</t>
         </is>
       </c>
       <c r="F469" t="inlineStr">
@@ -29507,7 +29507,7 @@
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F470" t="inlineStr">
@@ -29817,7 +29817,7 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F475" t="inlineStr">
@@ -29879,7 +29879,7 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F476" t="inlineStr">
@@ -30003,7 +30003,7 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>$6</t>
+          <t>$6,200,000</t>
         </is>
       </c>
       <c r="F478" t="inlineStr">
@@ -30065,7 +30065,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,000,000</t>
         </is>
       </c>
       <c r="F479" t="inlineStr">
@@ -30127,7 +30127,7 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>$21</t>
+          <t>$21,500,000</t>
         </is>
       </c>
       <c r="F480" t="inlineStr">
@@ -30187,7 +30187,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,000,000</t>
         </is>
       </c>
       <c r="F481" t="inlineStr">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>$7</t>
+          <t>$7,000,000</t>
         </is>
       </c>
       <c r="F482" t="inlineStr">
@@ -30311,7 +30311,7 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>$9</t>
+          <t>$9,300,000</t>
         </is>
       </c>
       <c r="F483" t="inlineStr">
@@ -30931,7 +30931,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>$160</t>
+          <t>$160,000,000</t>
         </is>
       </c>
       <c r="F493" t="inlineStr">
@@ -31179,7 +31179,7 @@
       </c>
       <c r="E497" t="inlineStr">
         <is>
-          <t>$130</t>
+          <t>$130,000,000</t>
         </is>
       </c>
       <c r="F497" t="inlineStr">
@@ -32667,7 +32667,7 @@
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>$100</t>
+          <t>$100,000,000</t>
         </is>
       </c>
       <c r="F521" t="inlineStr">
@@ -32977,7 +32977,7 @@
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>$80</t>
+          <t>$80,000,000</t>
         </is>
       </c>
       <c r="F526" t="inlineStr">
@@ -33287,7 +33287,7 @@
       </c>
       <c r="E531" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F531" t="inlineStr">
@@ -34029,7 +34029,7 @@
       </c>
       <c r="E543" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F543" t="inlineStr">
@@ -34399,7 +34399,7 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>$60</t>
+          <t>$60,000,000</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
@@ -34647,7 +34647,7 @@
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>$35</t>
+          <t>$35,000,000</t>
         </is>
       </c>
       <c r="F553" t="inlineStr">
@@ -34709,7 +34709,7 @@
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F554" t="inlineStr">
@@ -34833,7 +34833,7 @@
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F556" t="inlineStr">
@@ -34895,7 +34895,7 @@
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F557" t="inlineStr">
@@ -35019,7 +35019,7 @@
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>$18</t>
+          <t>$18,000,000</t>
         </is>
       </c>
       <c r="F559" t="inlineStr">
@@ -35205,7 +35205,7 @@
       </c>
       <c r="E562" t="inlineStr">
         <is>
-          <t>$65</t>
+          <t>$40,000,000</t>
         </is>
       </c>
       <c r="F562" t="inlineStr">
@@ -35391,7 +35391,7 @@
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F565" t="inlineStr">
@@ -35699,7 +35699,7 @@
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15,000,000</t>
         </is>
       </c>
       <c r="F570" t="inlineStr">
@@ -35945,7 +35945,7 @@
       </c>
       <c r="E574" t="inlineStr">
         <is>
-          <t>$35</t>
+          <t>$35,000,000</t>
         </is>
       </c>
       <c r="F574" t="inlineStr">
@@ -36379,7 +36379,7 @@
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$11,000,000</t>
         </is>
       </c>
       <c r="F581" t="inlineStr">
@@ -36441,7 +36441,7 @@
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>$39</t>
+          <t>$39,000,000</t>
         </is>
       </c>
       <c r="F582" t="inlineStr">
@@ -36625,7 +36625,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F585" t="inlineStr">
@@ -36749,7 +36749,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,500,000</t>
         </is>
       </c>
       <c r="F587" t="inlineStr">
@@ -36811,7 +36811,7 @@
       </c>
       <c r="E588" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F588" t="inlineStr">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>$35</t>
+          <t>$35,000,000</t>
         </is>
       </c>
       <c r="F592" t="inlineStr">
@@ -37307,7 +37307,7 @@
       </c>
       <c r="E596" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,500,000</t>
         </is>
       </c>
       <c r="F596" t="inlineStr">
@@ -37431,7 +37431,7 @@
       </c>
       <c r="E598" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,500,000</t>
         </is>
       </c>
       <c r="F598" t="inlineStr">
@@ -37679,7 +37679,7 @@
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,200,000</t>
         </is>
       </c>
       <c r="F602" t="inlineStr">
@@ -37741,7 +37741,7 @@
       </c>
       <c r="E603" t="inlineStr">
         <is>
-          <t>$34</t>
+          <t>$34,000,000</t>
         </is>
       </c>
       <c r="F603" t="inlineStr">
@@ -37803,7 +37803,7 @@
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F604" t="inlineStr">
@@ -37927,7 +37927,7 @@
       </c>
       <c r="E606" t="inlineStr">
         <is>
-          <t>$100</t>
+          <t>$100,000,000</t>
         </is>
       </c>
       <c r="F606" t="inlineStr">
@@ -38175,7 +38175,7 @@
       </c>
       <c r="E610" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,000,000</t>
         </is>
       </c>
       <c r="F610" t="inlineStr">
@@ -38299,7 +38299,7 @@
       </c>
       <c r="E612" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,000,000</t>
         </is>
       </c>
       <c r="F612" t="inlineStr">
@@ -38361,7 +38361,7 @@
       </c>
       <c r="E613" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15,800,000</t>
         </is>
       </c>
       <c r="F613" t="inlineStr">
@@ -38485,7 +38485,7 @@
       </c>
       <c r="E615" t="inlineStr">
         <is>
-          <t>$39</t>
+          <t>$39,000,000</t>
         </is>
       </c>
       <c r="F615" t="inlineStr">
@@ -38609,7 +38609,7 @@
       </c>
       <c r="E617" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,800,000</t>
         </is>
       </c>
       <c r="F617" t="inlineStr">
@@ -38733,7 +38733,7 @@
       </c>
       <c r="E619" t="inlineStr">
         <is>
-          <t>$4</t>
+          <t>$4,000,000</t>
         </is>
       </c>
       <c r="F619" t="inlineStr">
@@ -38857,7 +38857,7 @@
       </c>
       <c r="E621" t="inlineStr">
         <is>
-          <t>$50</t>
+          <t>$50,000,000</t>
         </is>
       </c>
       <c r="F621" t="inlineStr">
@@ -38919,7 +38919,7 @@
       </c>
       <c r="E622" t="inlineStr">
         <is>
-          <t>$1</t>
+          <t>$1,500,000</t>
         </is>
       </c>
       <c r="F622" t="inlineStr">
@@ -38981,7 +38981,7 @@
       </c>
       <c r="E623" t="inlineStr">
         <is>
-          <t>$19</t>
+          <t>$19,300,000</t>
         </is>
       </c>
       <c r="F623" t="inlineStr">
@@ -39043,7 +39043,7 @@
       </c>
       <c r="E624" t="inlineStr">
         <is>
-          <t>$1</t>
+          <t>$1,700,000</t>
         </is>
       </c>
       <c r="F624" t="inlineStr">
@@ -39105,7 +39105,7 @@
       </c>
       <c r="E625" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F625" t="inlineStr">
@@ -39167,7 +39167,7 @@
       </c>
       <c r="E626" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$11,000,000</t>
         </is>
       </c>
       <c r="F626" t="inlineStr">
@@ -39229,7 +39229,7 @@
       </c>
       <c r="E627" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15,500,000</t>
         </is>
       </c>
       <c r="F627" t="inlineStr">
@@ -39291,7 +39291,7 @@
       </c>
       <c r="E628" t="inlineStr">
         <is>
-          <t>$9</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F628" t="inlineStr">
@@ -39353,7 +39353,7 @@
       </c>
       <c r="E629" t="inlineStr">
         <is>
-          <t>$4</t>
+          <t>$4,000,000</t>
         </is>
       </c>
       <c r="F629" t="inlineStr">
@@ -39415,7 +39415,7 @@
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>$6</t>
+          <t>$6,000,000</t>
         </is>
       </c>
       <c r="F630" t="inlineStr">
@@ -39725,7 +39725,7 @@
       </c>
       <c r="E635" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>$13,150,000</t>
         </is>
       </c>
       <c r="F635" t="inlineStr">
@@ -39787,7 +39787,7 @@
       </c>
       <c r="E636" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F636" t="inlineStr">
@@ -40097,7 +40097,7 @@
       </c>
       <c r="E641" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F641" t="inlineStr">
@@ -40159,7 +40159,7 @@
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F642" t="inlineStr">
@@ -40221,7 +40221,7 @@
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>$4</t>
+          <t>$4,000,000</t>
         </is>
       </c>
       <c r="F643" t="inlineStr">
@@ -40283,7 +40283,7 @@
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>$2</t>
+          <t>$2,700,000</t>
         </is>
       </c>
       <c r="F644" t="inlineStr">
@@ -40469,7 +40469,7 @@
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>$38</t>
+          <t>$38,000,000</t>
         </is>
       </c>
       <c r="F647" t="inlineStr">
@@ -40531,7 +40531,7 @@
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,400,000</t>
         </is>
       </c>
       <c r="F648" t="inlineStr">
@@ -40593,7 +40593,7 @@
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>$7</t>
+          <t>$7,000,000</t>
         </is>
       </c>
       <c r="F649" t="inlineStr">
@@ -40655,7 +40655,7 @@
       </c>
       <c r="E650" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F650" t="inlineStr">
@@ -40779,7 +40779,7 @@
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>$18</t>
+          <t>$18,800,000</t>
         </is>
       </c>
       <c r="F652" t="inlineStr">
@@ -41027,7 +41027,7 @@
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>$1</t>
+          <t>$1,100,000</t>
         </is>
       </c>
       <c r="F656" t="inlineStr">
@@ -47161,7 +47161,7 @@
       </c>
       <c r="E755" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F755" t="inlineStr">
@@ -47223,7 +47223,7 @@
       </c>
       <c r="E756" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F756" t="inlineStr">
@@ -47905,7 +47905,7 @@
       </c>
       <c r="E767" t="inlineStr">
         <is>
-          <t>$45</t>
+          <t>$45,000,000</t>
         </is>
       </c>
       <c r="F767" t="inlineStr">
@@ -48091,7 +48091,7 @@
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,000,000</t>
         </is>
       </c>
       <c r="F770" t="inlineStr">
@@ -48277,7 +48277,7 @@
       </c>
       <c r="E773" t="inlineStr">
         <is>
-          <t>$59</t>
+          <t>$59,000,000</t>
         </is>
       </c>
       <c r="F773" t="inlineStr">
@@ -48339,7 +48339,7 @@
       </c>
       <c r="E774" t="inlineStr">
         <is>
-          <t>$100</t>
+          <t>$100,000,000</t>
         </is>
       </c>
       <c r="F774" t="inlineStr">
@@ -48401,7 +48401,7 @@
       </c>
       <c r="E775" t="inlineStr">
         <is>
-          <t>$9</t>
+          <t>$9,500,000</t>
         </is>
       </c>
       <c r="F775" t="inlineStr">
@@ -48525,7 +48525,7 @@
       </c>
       <c r="E777" t="inlineStr">
         <is>
-          <t>$12</t>
+          <t>$12,000,000</t>
         </is>
       </c>
       <c r="F777" t="inlineStr">
@@ -48649,7 +48649,7 @@
       </c>
       <c r="E779" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F779" t="inlineStr">
@@ -48835,7 +48835,7 @@
       </c>
       <c r="E782" t="inlineStr">
         <is>
-          <t>$15</t>
+          <t>$15,000,000</t>
         </is>
       </c>
       <c r="F782" t="inlineStr">
@@ -48959,7 +48959,7 @@
       </c>
       <c r="E784" t="inlineStr">
         <is>
-          <t>$11</t>
+          <t>$11,000,000</t>
         </is>
       </c>
       <c r="F784" t="inlineStr">
@@ -49207,7 +49207,7 @@
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>$17</t>
+          <t>$17,300,000</t>
         </is>
       </c>
       <c r="F788" t="inlineStr">
@@ -49331,7 +49331,7 @@
       </c>
       <c r="E790" t="inlineStr">
         <is>
-          <t>$18</t>
+          <t>$18,000,000</t>
         </is>
       </c>
       <c r="F790" t="inlineStr">
@@ -49393,7 +49393,7 @@
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F791" t="inlineStr">
@@ -49455,7 +49455,7 @@
       </c>
       <c r="E792" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F792" t="inlineStr">
@@ -49701,7 +49701,7 @@
       </c>
       <c r="E796" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F796" t="inlineStr">
@@ -49763,7 +49763,7 @@
       </c>
       <c r="E797" t="inlineStr">
         <is>
-          <t>$1</t>
+          <t>$1,500,000</t>
         </is>
       </c>
       <c r="F797" t="inlineStr">
@@ -49825,7 +49825,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F798" t="inlineStr">
@@ -49887,7 +49887,7 @@
       </c>
       <c r="E799" t="inlineStr">
         <is>
-          <t>$25</t>
+          <t>$25,000,000</t>
         </is>
       </c>
       <c r="F799" t="inlineStr">
@@ -49949,7 +49949,7 @@
       </c>
       <c r="E800" t="inlineStr">
         <is>
-          <t>$50</t>
+          <t>$50,000,000</t>
         </is>
       </c>
       <c r="F800" t="inlineStr">
@@ -50073,7 +50073,7 @@
       </c>
       <c r="E802" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F802" t="inlineStr">
@@ -50259,7 +50259,7 @@
       </c>
       <c r="E805" t="inlineStr">
         <is>
-          <t>$9</t>
+          <t>$9,000,000</t>
         </is>
       </c>
       <c r="F805" t="inlineStr">
@@ -50321,7 +50321,7 @@
       </c>
       <c r="E806" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F806" t="inlineStr">
@@ -50383,7 +50383,7 @@
       </c>
       <c r="E807" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$20,000,000</t>
         </is>
       </c>
       <c r="F807" t="inlineStr">
@@ -50445,7 +50445,7 @@
       </c>
       <c r="E808" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>$10,000,000</t>
         </is>
       </c>
       <c r="F808" t="inlineStr">
@@ -50507,7 +50507,7 @@
       </c>
       <c r="E809" t="inlineStr">
         <is>
-          <t>$30</t>
+          <t>$30,000,000</t>
         </is>
       </c>
       <c r="F809" t="inlineStr">
@@ -50569,7 +50569,7 @@
       </c>
       <c r="E810" t="inlineStr">
         <is>
-          <t>$5</t>
+          <t>$5,000,000</t>
         </is>
       </c>
       <c r="F810" t="inlineStr">
@@ -50755,7 +50755,7 @@
       </c>
       <c r="E813" t="inlineStr">
         <is>
-          <t>$3</t>
+          <t>$3,000,000</t>
         </is>
       </c>
       <c r="F813" t="inlineStr">
@@ -50879,7 +50879,7 @@
       </c>
       <c r="E815" t="inlineStr">
         <is>
-          <t>$8</t>
+          <t>$8,000,000</t>
         </is>
       </c>
       <c r="F815" t="inlineStr">
@@ -51065,7 +51065,7 @@
       </c>
       <c r="E818" t="inlineStr">
         <is>
-          <t>$40</t>
+          <t>$40,000,000</t>
         </is>
       </c>
       <c r="F818" t="inlineStr">
@@ -52303,7 +52303,7 @@
       </c>
       <c r="E838" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>$12,000,000</t>
         </is>
       </c>
       <c r="F838" t="inlineStr">
@@ -52489,7 +52489,7 @@
       </c>
       <c r="E841" t="inlineStr">
         <is>
-          <t>$18</t>
+          <t>$18,600,000</t>
         </is>
       </c>
       <c r="F841" t="inlineStr">

</xml_diff>